<commit_message>
Array Question 1 Completed
</commit_message>
<xml_diff>
--- a/dsa_questions_all_450_enhanced.xlsx
+++ b/dsa_questions_all_450_enhanced.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding word\js\Data Science Algorithm From Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DAC2BB8-C2CB-4CC0-8431-2C69801BEC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6B0AE2-AB40-4BCE-A2FD-F3B3DFE4A0C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7872" yWindow="0" windowWidth="15264" windowHeight="12336" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2283" uniqueCount="1285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2285" uniqueCount="1287">
   <si>
     <t>DSA Questions Summary - Complete Edition (450 Questions)</t>
   </si>
@@ -3893,6 +3893,12 @@
   </si>
   <si>
     <t>Questions</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -3985,7 +3991,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4003,6 +4009,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4612,7 +4621,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E451"/>
+  <dimension ref="A1:F451"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" style="4" customWidth="1"/>
@@ -4620,10 +4629,11 @@
     <col min="3" max="3" width="95" style="4" customWidth="1"/>
     <col min="4" max="4" width="22" style="4" customWidth="1"/>
     <col min="5" max="5" width="15" style="4" customWidth="1"/>
-    <col min="6" max="16384" width="8.6640625" style="4"/>
+    <col min="6" max="6" width="28.21875" style="4" customWidth="1"/>
+    <col min="7" max="16384" width="8.6640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>1284</v>
       </c>
@@ -4639,8 +4649,11 @@
       <c r="E1" s="3" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+      <c r="F1" s="4" t="s">
+        <v>1285</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -4656,8 +4669,11 @@
       <c r="E2" s="5" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="66" x14ac:dyDescent="0.3">
+      <c r="F2" s="9" t="s">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="66" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>37</v>
       </c>
@@ -4674,7 +4690,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>40</v>
       </c>
@@ -4691,7 +4707,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>43</v>
       </c>
@@ -4708,7 +4724,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>46</v>
       </c>
@@ -4725,7 +4741,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>49</v>
       </c>
@@ -4742,7 +4758,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>52</v>
       </c>
@@ -4759,7 +4775,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>55</v>
       </c>
@@ -4776,7 +4792,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>58</v>
       </c>
@@ -4793,7 +4809,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>61</v>
       </c>
@@ -4810,7 +4826,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>64</v>
       </c>
@@ -4827,7 +4843,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>68</v>
       </c>
@@ -4844,7 +4860,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>71</v>
       </c>
@@ -4861,7 +4877,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="52.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>74</v>
       </c>
@@ -4878,7 +4894,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>77</v>
       </c>

</xml_diff>

<commit_message>
Array--> Question 3 Contains Duplicate ✅Solved
</commit_message>
<xml_diff>
--- a/dsa_questions_all_450_enhanced.xlsx
+++ b/dsa_questions_all_450_enhanced.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding word\js\Data Science Algorithm From Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB49BF55-AF91-46BF-9662-24A702249A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D403360D-5AF5-4371-938D-84FFECEDBBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2286" uniqueCount="1287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2287" uniqueCount="1287">
   <si>
     <t>DSA Questions Summary - Complete Edition (450 Questions)</t>
   </si>
@@ -4709,6 +4709,9 @@
       <c r="E4" s="5" t="s">
         <v>36</v>
       </c>
+      <c r="F4" s="8" t="s">
+        <v>1286</v>
+      </c>
     </row>
     <row r="5" spans="1:6" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">

</xml_diff>